<commit_message>
Polish ELP export layout and keep in-album photo order.
Persist photo_file_order, slim empty ELP photo slots, refresh TOC via Word, and cache embed JPEGs so export stays fast. Version stays 1.4.0.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/templates/standard sheet/标准库.xlsx
+++ b/templates/standard sheet/标准库.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10821"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10914"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D571FD64-9739-A849-8881-BF464E008A4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{883BB844-FD85-C44B-B28C-AC1E3CD1EC48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="27880" windowHeight="17280" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -67,7 +67,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="975" uniqueCount="496">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="980" uniqueCount="501">
   <si>
     <t>标准号</t>
   </si>
@@ -1877,6 +1877,27 @@
   </si>
   <si>
     <t>环境温湿度</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Q/JLY J7111029E-2024①</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>5.1.8</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>反极性</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>样品需满足功能状态C，且在反极性时，不允许激活零部件的重要安全功能。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>严重程度一：满足功能状态C，在反极性时，未激活零部件的重要安全功能。
+严重程度二：满足功能状态C，在反极性时，未激活零部件的重要安全功能。</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -2361,7 +2382,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:S102"/>
+  <dimension ref="A1:S103"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="80" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="24.83203125" style="1" customWidth="1"/>
@@ -6111,6 +6132,23 @@
         <v>45925.581400462965</v>
       </c>
     </row>
+    <row r="103" spans="1:17" ht="80" customHeight="1">
+      <c r="A103" s="1" t="s">
+        <v>496</v>
+      </c>
+      <c r="B103" s="1" t="s">
+        <v>497</v>
+      </c>
+      <c r="C103" s="1" t="s">
+        <v>498</v>
+      </c>
+      <c r="I103" s="2" t="s">
+        <v>499</v>
+      </c>
+      <c r="K103" s="2" t="s">
+        <v>500</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="14">
     <mergeCell ref="O61:O66"/>

</xml_diff>